<commit_message>
feat(F-NAR-019): TREE-COL-028 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-028.xlsx
+++ b/stories/arbres/TREE-COL-028.xlsx
@@ -2348,17 +2348,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>La boîte du goûter est près de la casserole. Le couvercle est tiède, un peu collant. Je la prends ! Nina avance la main. La chaleur la fait reculer. Maman parle du lait, sans se presser. Nina attend la fin de la phrase. Le goûter, s'il te plaît. Le voilà, il a refroidi. Merci. Tu as demandé au bon moment. La boîte glisse dans le cartable, toc. Une odeur de cacao reste sur le couvercle.</t>
+          <t>La boîte du goûter est près de la casserole. Le couvercle est tiède, un peu collant. Je la prends ! Nina avance la main. La chaleur la fait reculer. Maman parle du lait, sans se presser. Nina attend la fin de la phrase. Le goûter, s'il te plaît. Le voilà, il a refroidi. Merci. Je t'ai entendue, là. La boîte glisse dans le cartable, toc. Une odeur de cacao reste sur le couvercle.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La boîte du goûter est près de la casserole. Le couvercle est tiède, un peu collant. Je la prends ! Nina avance la main. La chaleur la fait reculer. Maman parle du lait, sans se presser. Nina attend la fin de la phrase. Le goûter, s'il te plaît. Le voilà, il a refroidi. Merci. Tu as demandé au bon moment. La boîte glisse dans le cartable, toc. Une odeur de cacao reste sur le couvercle.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;La boîte du goûter est près de la casserole. Le couvercle est tiède, un peu collant. Je la prends ! Nina avance la main. La chaleur la fait reculer. Maman parle du lait, sans se presser. Nina attend la fin de la phrase. Le goûter, s'il te plaît. Le voilà, il a refroidi. Merci. Je t'ai entendue, là. La boîte glisse dans le cartable, toc. Une odeur de cacao reste sur le couvercle.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;La boîte du goûter est près de la casserole. Le couvercle est tiède, un peu collant. Je la prends ! Nina avance la main. La chaleur la fait reculer. Maman parle du lait, sans se presser. Nina attend la fin de la phrase. Le goûter, s'il te plaît. Le voilà, il a refroidi. Merci. Tu as demandé au bon moment. La boîte glisse dans le cartable, toc. Une odeur de cacao reste sur le couvercle.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;La boîte du goûter est près de la casserole. Le couvercle est tiède, un peu collant. Je la prends ! Nina avance la main. La chaleur la fait reculer. Maman parle du lait, sans se presser. Nina attend la fin de la phrase. Le goûter, s'il te plaît. Le voilà, il a refroidi. Merci. Je t'ai entendue, là. La boîte glisse dans le cartable, toc. Une odeur de cacao reste sur le couvercle.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
 enfant-f|Le goûter, s'il te plaît.
 maman|Le voilà, il a refroidi.
 enfant-f|Merci.
-papa|Tu as demandé au bon moment.
+papa|Je t'ai entendue, là.
 narrateur|La boîte glisse dans le cartable, toc.
 narrateur|Une odeur de cacao reste sur le couvercle.</t>
         </is>
@@ -2923,17 +2923,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Nina marche sur le chemin, le cartable au dos. La boîte fait un petit toc, à chaque pas. Il est à moi. Tu l'as demandé. Bravo, Nina. Derrière elle, la vitre de la cuisine est nette. Une miette dorée brille sur la boucle. Le rond de manche n'est plus un nuage.</t>
+          <t>Nina marche sur le chemin, le cartable au dos. La boîte fait un petit toc, à chaque pas. Il est à moi. Il tient bien, au dos. Bravo, Nina. Derrière elle, la vitre de la cuisine est nette. Une miette dorée brille sur la boucle. Le rond de manche n'est plus un nuage.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina marche sur le chemin, le cartable au dos. La boîte fait un petit toc, à chaque pas. Il est à moi. Tu l'as demandé. Bravo, Nina. Derrière elle, la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; de la cuisine est nette. Une miette dorée brille sur la boucle. Le rond de manche n'est plus un nuage.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina marche sur le chemin, le cartable au dos. La boîte fait un petit toc, à chaque pas. Il est à moi. Il tient bien, au dos. Bravo, Nina. Derrière elle, la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; de la cuisine est nette. Une miette dorée brille sur la boucle. Le rond de manche n'est plus un nuage.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina marche sur le chemin, le cartable au dos. La boîte fait un petit toc, à chaque pas. Il est à moi. Tu l'as demandé. Bravo, Nina. Derrière elle, la &lt;emphasis&gt;vitre&lt;/emphasis&gt; de la cuisine est nette. Une miette dorée brille sur la boucle. Le rond de manche n'est plus un nuage.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina marche sur le chemin, le cartable au dos. La boîte fait un petit toc, à chaque pas. Il est à moi. Il tient bien, au dos. Bravo, Nina. Derrière elle, la &lt;emphasis&gt;vitre&lt;/emphasis&gt; de la cuisine est nette. Une miette dorée brille sur la boucle. Le rond de manche n'est plus un nuage.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3074,7 +3074,7 @@
           <t>narrateur|Nina marche sur le chemin, le cartable au dos.
 narrateur|La boîte fait un petit toc, à chaque pas.
 enfant-f|Il est à moi.
-papa|Tu l'as demandé.
+papa|Il tient bien, au dos.
 maman|Bravo, Nina.
 narrateur|Derrière elle, la vitre de la cuisine est nette.
 narrateur|Une miette dorée brille sur la boucle.
@@ -3296,17 +3296,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Nina s'assoit près du bol, le cartable contre elle. La boîte est tiède, au fond. On partira plus tard. Oui. Merci d'avoir attendu. Un carré de soleil a fini de sécher le verre. Plus de voix dans le cacao. Ce jaune-là est devenu mat, paisible.</t>
+          <t>Nina s'assoit près du bol, le cartable contre elle. La boîte est tiède, au fond. On partira plus tard. Oui. Merci, on n'est pas pressés. Un carré de soleil a fini de sécher le verre. Plus de voix dans le cacao. Ce jaune-là est devenu mat, paisible.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina s'assoit près du bol, le cartable contre elle. La boîte est tiède, au fond. On partira plus tard. Oui. Merci d'avoir attendu. Un carré de soleil a fini de sécher le verre. Plus de voix dans le cacao. Ce jaune-là est devenu mat, paisible.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina s'assoit près du bol, le cartable contre elle. La boîte est tiède, au fond. On partira plus tard. Oui. Merci, on n'est pas pressés. Un carré de soleil a fini de sécher le verre. Plus de voix dans le cacao. Ce jaune-là est devenu mat, paisible.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina s'assoit près du bol, le cartable contre elle. La boîte est tiède, au fond. On partira plus tard. Oui. Merci d'avoir attendu. Un carré de soleil a fini de sécher le verre. Plus de voix dans le cacao. Ce jaune-là est devenu mat, paisible.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina s'assoit près du bol, le cartable contre elle. La boîte est tiède, au fond. On partira plus tard. Oui. Merci, on n'est pas pressés. Un carré de soleil a fini de sécher le verre. Plus de voix dans le cacao. Ce jaune-là est devenu mat, paisible.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3448,7 +3448,7 @@
 narrateur|La boîte est tiède, au fond.
 enfant-f|On partira plus tard.
 maman|Oui.
-papa|Merci d'avoir attendu.
+papa|Merci, on n'est pas pressés.
 narrateur|Un carré de soleil a fini de sécher le verre.
 narrateur|Plus de voix dans le cacao.
 narrateur|Ce jaune-là est devenu mat, paisible.</t>
@@ -4429,17 +4429,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Sur le chemin, la poche frotte un peu le dos de Nina. Le dessin est là, droit. La maison jaune vient avec moi. Je l'ai vue. Merci de l'avoir glissée sans la froisser. Le toit de la classe grandit. La vitre, derrière, garde un ovale clair. Plus de papier collé au verre.</t>
+          <t>Sur le chemin, la poche frotte un peu le dos de Nina. Le dessin est là, droit. La maison jaune vient avec moi. Je l'ai vue. Merci, le papier n'a pas de pli. Le toit de la classe grandit. La vitre, derrière, garde un ovale clair. Plus de papier collé au verre.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le chemin, la poche frotte un peu le dos de Nina. Le dessin est là, droit. La maison jaune vient avec moi. Je l'ai vue. Merci de l'avoir glissée sans la froisser. Le toit de la classe grandit. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt;, derrière, garde un ovale clair. Plus de papier collé au verre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le chemin, la poche frotte un peu le dos de Nina. Le dessin est là, droit. La maison jaune vient avec moi. Je l'ai vue. Merci, le papier n'a pas de pli. Le toit de la classe grandit. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt;, derrière, garde un ovale clair. Plus de papier collé au verre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le chemin, la poche frotte un peu le dos de Nina. Le dessin est là, droit. La maison jaune vient avec moi. Je l'ai vue. Merci de l'avoir glissée sans la froisser. Le toit de la classe grandit. La &lt;emphasis&gt;vitre&lt;/emphasis&gt;, derrière, garde un ovale clair. Plus de papier collé au verre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le chemin, la poche frotte un peu le dos de Nina. Le dessin est là, droit. La maison jaune vient avec moi. Je l'ai vue. Merci, le papier n'a pas de pli. Le toit de la classe grandit. La &lt;emphasis&gt;vitre&lt;/emphasis&gt;, derrière, garde un ovale clair. Plus de papier collé au verre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4581,7 +4581,7 @@
 narrateur|Le dessin est là, droit.
 enfant-f|La maison jaune vient avec moi.
 maman|Je l'ai vue.
-papa|Merci de l'avoir glissée sans la froisser.
+papa|Merci, le papier n'a pas de pli.
 narrateur|Le toit de la classe grandit.
 narrateur|La vitre, derrière, garde un ovale clair.
 narrateur|Plus de papier collé au verre.</t>
@@ -4801,17 +4801,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Nina pose le cartable près du bol. Le coin du dessin n'est plus mouillé. Elle est droite, ma maison. Oui. Merci d'avoir lissé sans casser. La vitre n'a plus de larmes. Un rond clair reste, comme une fenêtre dans la fenêtre. Le chemin attend, sans se presser.</t>
+          <t>Nina pose le cartable près du bol. Le coin du dessin n'est plus mouillé. Elle est droite, ma maison. Oui. Ta maison est droite, merci. La vitre n'a plus de larmes. Un rond clair reste, comme une fenêtre dans la fenêtre. Le chemin attend, sans se presser.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina pose le cartable près du bol. Le coin du dessin n'est plus mouillé. Elle est droite, ma maison. Oui. Merci d'avoir lissé sans casser. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; n'a plus de larmes. Un rond clair reste, comme une fenêtre dans la fenêtre. Le chemin attend, sans se presser.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina pose le cartable près du bol. Le coin du dessin n'est plus mouillé. Elle est droite, ma maison. Oui. Ta maison est droite, merci. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; n'a plus de larmes. Un rond clair reste, comme une fenêtre dans la fenêtre. Le chemin attend, sans se presser.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina pose le cartable près du bol. Le coin du dessin n'est plus mouillé. Elle est droite, ma maison. Oui. Merci d'avoir lissé sans casser. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; n'a plus de larmes. Un rond clair reste, comme une fenêtre dans la fenêtre. Le chemin attend, sans se presser.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina pose le cartable près du bol. Le coin du dessin n'est plus mouillé. Elle est droite, ma maison. Oui. Ta maison est droite, merci. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; n'a plus de larmes. Un rond clair reste, comme une fenêtre dans la fenêtre. Le chemin attend, sans se presser.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4953,7 +4953,7 @@
 narrateur|Le coin du dessin n'est plus mouillé.
 enfant-f|Elle est droite, ma maison.
 papa|Oui.
-maman|Merci d'avoir lissé sans casser.
+maman|Ta maison est droite, merci.
 narrateur|La vitre n'a plus de larmes.
 narrateur|Un rond clair reste, comme une fenêtre dans la fenêtre.
 narrateur|Le chemin attend, sans se presser.</t>
@@ -5934,17 +5934,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Nina passe l'ovale, le cartable au dos. Le torchon reste sur la chaise, taché d'un peu de jaune. Je vois le chemin. Nous aussi. Merci d'avoir guidé le geste. L'ovale encadre la haie, puis se perd. Le toit de la classe est net. Le cacao n'embue plus rien.</t>
+          <t>Nina passe l'ovale, le cartable au dos. Le torchon reste sur la chaise, taché d'un peu de jaune. Je vois le chemin. Nous aussi. Merci, on a vu le chemin ensemble. L'ovale encadre la haie, puis se perd. Le toit de la classe est net. Le cacao n'embue plus rien.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina passe l'ovale, le cartable au dos. Le torchon reste sur la chaise, taché d'un peu de jaune. Je vois le chemin. Nous aussi. Merci d'avoir guidé le geste. L'ovale encadre la haie, puis se perd. Le toit de la classe est net. Le cacao n'embue plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina passe l'ovale, le cartable au dos. Le torchon reste sur la chaise, taché d'un peu de jaune. Je vois le chemin. Nous aussi. Merci, on a vu le chemin ensemble. L'ovale encadre la haie, puis se perd. Le toit de la classe est net. Le cacao n'embue plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina passe l'ovale, le cartable au dos. Le torchon reste sur la chaise, taché d'un peu de jaune. Je vois le chemin. Nous aussi. Merci d'avoir guidé le geste. L'ovale encadre la haie, puis se perd. Le toit de la classe est net. Le cacao n'embue plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina passe l'ovale, le cartable au dos. Le torchon reste sur la chaise, taché d'un peu de jaune. Je vois le chemin. Nous aussi. Merci, on a vu le chemin ensemble. L'ovale encadre la haie, puis se perd. Le toit de la classe est net. Le cacao n'embue plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6086,7 +6086,7 @@
 narrateur|Le torchon reste sur la chaise, taché d'un peu de jaune.
 enfant-f|Je vois le chemin.
 papa|Nous aussi.
-maman|Merci d'avoir guidé le geste.
+maman|Merci, on a vu le chemin ensemble.
 narrateur|L'ovale encadre la haie, puis se perd.
 narrateur|Le toit de la classe est net.
 narrateur|Le cacao n'embue plus rien.</t>
@@ -6307,17 +6307,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Nina n'a pas frotté. Le chemin était là, sans elle. Le torchon se repose. Oui. Merci d'avoir regardé d'abord. Le torchon sent le four, sur la chaise. La vitre est un miroir, sans travail. Le cartable attend près du bol, prêt.</t>
+          <t>Nina n'a pas frotté. Le chemin était là, sans elle. Le torchon se repose. Oui. Merci, tes yeux ont suffi. Le torchon sent le four, sur la chaise. La vitre est un miroir, sans travail. Le cartable attend près du bol, prêt.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina n'a pas frotté. Le chemin était là, sans elle. Le torchon se repose. Oui. Merci d'avoir regardé d'abord. Le torchon sent le four, sur la chaise. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; est un miroir, sans travail. Le cartable attend près du bol, prêt.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina n'a pas frotté. Le chemin était là, sans elle. Le torchon se repose. Oui. Merci, tes yeux ont suffi. Le torchon sent le four, sur la chaise. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; est un miroir, sans travail. Le cartable attend près du bol, prêt.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina n'a pas frotté. Le chemin était là, sans elle. Le torchon se repose. Oui. Merci d'avoir regardé d'abord. Le torchon sent le four, sur la chaise. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; est un miroir, sans travail. Le cartable attend près du bol, prêt.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina n'a pas frotté. Le chemin était là, sans elle. Le torchon se repose. Oui. Merci, tes yeux ont suffi. Le torchon sent le four, sur la chaise. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; est un miroir, sans travail. Le cartable attend près du bol, prêt.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6459,7 +6459,7 @@
 narrateur|Le chemin était là, sans elle.
 enfant-f|Le torchon se repose.
 maman|Oui.
-papa|Merci d'avoir regardé d'abord.
+papa|Merci, tes yeux ont suffi.
 narrateur|Le torchon sent le four, sur la chaise.
 narrateur|La vitre est un miroir, sans travail.
 narrateur|Le cartable attend près du bol, prêt.</t>
@@ -6678,17 +6678,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Le torchon est sur le dossier, loin de la lampe. Le cartable dort contre le verre. Le jaune fait une lune. Je la vois. Merci d'avoir posé le tissu ailleurs. La buée tient autour de l'ovale, sans le manger. Le chemin de l'école est une ligne noire. La casserole est vide, tiède.</t>
+          <t>Le torchon est sur le dossier, loin de la lampe. Le cartable dort contre le verre. Le jaune fait une lune. Je la vois. Merci, la lampe reste libre. La buée tient autour de l'ovale, sans le manger. Le chemin de l'école est une ligne noire. La casserole est vide, tiède.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le torchon est sur le dossier, loin de la lampe. Le cartable dort contre le verre. Le jaune fait une lune. Je la vois. Merci d'avoir posé le tissu ailleurs. La buée tient autour de l'ovale, sans le manger. Le chemin de l'école est une ligne noire. La casserole est vide, tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le torchon est sur le dossier, loin de la lampe. Le cartable dort contre le verre. Le jaune fait une lune. Je la vois. Merci, la lampe reste libre. La buée tient autour de l'ovale, sans le manger. Le chemin de l'école est une ligne noire. La casserole est vide, tiède.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le torchon est sur le dossier, loin de la lampe. Le cartable dort contre le verre. Le jaune fait une lune. Je la vois. Merci d'avoir posé le tissu ailleurs. La buée tient autour de l'ovale, sans le manger. Le chemin de l'école est une ligne noire. La casserole est vide, tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le torchon est sur le dossier, loin de la lampe. Le cartable dort contre le verre. Le jaune fait une lune. Je la vois. Merci, la lampe reste libre. La buée tient autour de l'ovale, sans le manger. Le chemin de l'école est une ligne noire. La casserole est vide, tiède.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6830,7 +6830,7 @@
 narrateur|Le cartable dort contre le verre.
 enfant-f|Le jaune fait une lune.
 papa|Je la vois.
-maman|Merci d'avoir posé le tissu ailleurs.
+maman|Merci, la lampe reste libre.
 narrateur|La buée tient autour de l'ovale, sans le manger.
 narrateur|Le chemin de l'école est une ligne noire.
 narrateur|La casserole est vide, tiède.</t>
@@ -8195,17 +8195,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Nina marche, la boîte au dos, toc, toc. La feuille reste au crochet, comme un ticket oublié. Mon cartable ne glisse plus. La courroie est sèche. Merci d'avoir fermé avant de courir. Les dalles ne sont plus des cuillères. Le chemin brille, puis devient poussière claire. Le jardin reste derrière, mouillé et calme.</t>
+          <t>Nina marche, la boîte au dos, toc, toc. La feuille reste au crochet, comme un ticket oublié. Mon cartable ne glisse plus. La courroie est sèche. Merci, la fermeture tient. Les dalles ne sont plus des cuillères. Le chemin brille, puis devient poussière claire. Le jardin reste derrière, mouillé et calme.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina marche, la boîte au dos, toc, toc. La feuille reste au crochet, comme un ticket oublié. Mon cartable ne glisse plus. La courroie est sèche. Merci d'avoir fermé avant de courir. Les dalles ne sont plus des cuillères. Le chemin brille, puis devient poussière claire. Le jardin reste derrière, mouillé et calme.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina marche, la boîte au dos, toc, toc. La feuille reste au crochet, comme un ticket oublié. Mon cartable ne glisse plus. La courroie est sèche. Merci, la fermeture tient. Les dalles ne sont plus des cuillères. Le chemin brille, puis devient poussière claire. Le jardin reste derrière, mouillé et calme.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina marche, la boîte au dos, toc, toc. La feuille reste au crochet, comme un ticket oublié. Mon cartable ne glisse plus. La courroie est sèche. Merci d'avoir fermé avant de courir. Les dalles ne sont plus des cuillères. Le chemin brille, puis devient poussière claire. Le jardin reste derrière, mouillé et calme.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina marche, la boîte au dos, toc, toc. La feuille reste au crochet, comme un ticket oublié. Mon cartable ne glisse plus. La courroie est sèche. Merci, la fermeture tient. Les dalles ne sont plus des cuillères. Le chemin brille, puis devient poussière claire. Le jardin reste derrière, mouillé et calme.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8347,7 +8347,7 @@
 narrateur|La feuille reste au crochet, comme un ticket oublié.
 enfant-f|Mon cartable ne glisse plus.
 papa|La courroie est sèche.
-maman|Merci d'avoir fermé avant de courir.
+maman|Merci, la fermeture tient.
 narrateur|Les dalles ne sont plus des cuillères.
 narrateur|Le chemin brille, puis devient poussière claire.
 narrateur|Le jardin reste derrière, mouillé et calme.</t>
@@ -8568,17 +8568,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>L'abeille a quitté le thym. Nina tient le cartable à l'ombre du mur. Le goûter est tiède. Oui. Merci d'avoir attendu l'abeille. La table du jardin est sèche, presque blanche. Le couvercle sent l'herbe et le soleil. Le chemin, plus loin, ne dit rien.</t>
+          <t>L'abeille a quitté le thym. Nina tient le cartable à l'ombre du mur. Le goûter est tiède. Oui. Merci, l'abeille est partie. La table du jardin est sèche, presque blanche. Le couvercle sent l'herbe et le soleil. Le chemin, plus loin, ne dit rien.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'abeille a quitté le thym. Nina tient le cartable à l'ombre du mur. Le goûter est tiède. Oui. Merci d'avoir attendu l'abeille. La table du jardin est sèche, presque blanche. Le couvercle sent l'herbe et le soleil. Le chemin, plus loin, ne dit rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'abeille a quitté le thym. Nina tient le cartable à l'ombre du mur. Le goûter est tiède. Oui. Merci, l'abeille est partie. La table du jardin est sèche, presque blanche. Le couvercle sent l'herbe et le soleil. Le chemin, plus loin, ne dit rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'abeille a quitté le thym. Nina tient le cartable à l'ombre du mur. Le goûter est tiède. Oui. Merci d'avoir attendu l'abeille. La table du jardin est sèche, presque blanche. Le couvercle sent l'herbe et le soleil. Le chemin, plus loin, ne dit rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'abeille a quitté le thym. Nina tient le cartable à l'ombre du mur. Le goûter est tiède. Oui. Merci, l'abeille est partie. La table du jardin est sèche, presque blanche. Le couvercle sent l'herbe et le soleil. Le chemin, plus loin, ne dit rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8720,7 +8720,7 @@
 narrateur|Nina tient le cartable à l'ombre du mur.
 enfant-f|Le goûter est tiède.
 maman|Oui.
-papa|Merci d'avoir attendu l'abeille.
+papa|Merci, l'abeille est partie.
 narrateur|La table du jardin est sèche, presque blanche.
 narrateur|Le couvercle sent l'herbe et le soleil.
 narrateur|Le chemin, plus loin, ne dit rien.</t>
@@ -8940,17 +8940,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Le cartable est rentré, la boîte dedans. Le crochet de la porte est vide. Une étoile dans la goutte. Je la vois. Merci d'avoir demandé le décrochage. Le carré jaune a quitté la porte. Il est dans la cuisine, près des clés. Le jardin respire, sans le sac.</t>
+          <t>Le cartable est rentré, la boîte dedans. Le crochet de la porte est vide. Une étoile dans la goutte. Je la vois. Merci, Nina. Le carré jaune a quitté la porte. Il est dans la cuisine, près des clés. Le jardin respire, sans le sac.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable est rentré, la boîte dedans. Le crochet de la porte est vide. Une étoile dans la goutte. Je la vois. Merci d'avoir demandé le décrochage. Le carré jaune a quitté la porte. Il est dans la cuisine, près des clés. Le jardin respire, sans le sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable est rentré, la boîte dedans. Le crochet de la porte est vide. Une étoile dans la goutte. Je la vois. Merci, Nina. Le carré jaune a quitté la porte. Il est dans la cuisine, près des clés. Le jardin respire, sans le sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable est rentré, la boîte dedans. Le crochet de la porte est vide. Une étoile dans la goutte. Je la vois. Merci d'avoir demandé le décrochage. Le carré jaune a quitté la porte. Il est dans la cuisine, près des clés. Le jardin respire, sans le sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable est rentré, la boîte dedans. Le crochet de la porte est vide. Une étoile dans la goutte. Je la vois. Merci, Nina. Le carré jaune a quitté la porte. Il est dans la cuisine, près des clés. Le jardin respire, sans le sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9092,7 +9092,7 @@
 narrateur|Le crochet de la porte est vide.
 enfant-f|Une étoile dans la goutte.
 papa|Je la vois.
-maman|Merci d'avoir demandé le décrochage.
+maman|Merci, Nina.
 narrateur|Le carré jaune a quitté la porte.
 narrateur|Il est dans la cuisine, près des clés.
 narrateur|Le jardin respire, sans le sac.</t>
@@ -9699,17 +9699,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Nina marche, le dessin au chaud dans la poche. L'oiseau a quitté la haie. Je lui ai dit bonjour. Il a dû entendre. Merci d'avoir gardé le papier. Une goutte reste au milieu du chemin, puis sèche. Le thym colle aux doigts. Le jaune avance, sans voler.</t>
+          <t>Nina marche, le dessin au chaud dans la poche. L'oiseau a quitté la haie. Je lui ai dit bonjour. Il a dû entendre. Merci, le papier est au chaud. Une goutte reste au milieu du chemin, puis sèche. Le thym colle aux doigts. Le jaune avance, sans voler.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina marche, le dessin au chaud dans la poche. L'oiseau a quitté la haie. Je lui ai dit bonjour. Il a dû entendre. Merci d'avoir gardé le papier. Une goutte reste au milieu du chemin, puis sèche. Le thym colle aux doigts. Le jaune avance, sans voler.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina marche, le dessin au chaud dans la poche. L'oiseau a quitté la haie. Je lui ai dit bonjour. Il a dû entendre. Merci, le papier est au chaud. Une goutte reste au milieu du chemin, puis sèche. Le thym colle aux doigts. Le jaune avance, sans voler.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina marche, le dessin au chaud dans la poche. L'oiseau a quitté la haie. Je lui ai dit bonjour. Il a dû entendre. Merci d'avoir gardé le papier. Une goutte reste au milieu du chemin, puis sèche. Le thym colle aux doigts. Le jaune avance, sans voler.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina marche, le dessin au chaud dans la poche. L'oiseau a quitté la haie. Je lui ai dit bonjour. Il a dû entendre. Merci, le papier est au chaud. Une goutte reste au milieu du chemin, puis sèche. Le thym colle aux doigts. Le jaune avance, sans voler.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9851,7 +9851,7 @@
 narrateur|L'oiseau a quitté la haie.
 enfant-f|Je lui ai dit bonjour.
 maman|Il a dû entendre.
-papa|Merci d'avoir gardé le papier.
+papa|Merci, le papier est au chaud.
 narrateur|Une goutte reste au milieu du chemin, puis sèche.
 narrateur|Le thym colle aux doigts.
 narrateur|Le jaune avance, sans voler.</t>
@@ -10070,17 +10070,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>La veine d'herbe reste sur le papier, dans la poche. Nina s'assoit sur le seuil. C'est son voyage. Oui. Merci de l'avoir laissée. La vitre de la porte montre le banc, net. Le cartable est chaud, contre la jambe. Le chemin attend, large et pâle.</t>
+          <t>La veine d'herbe reste sur le papier, dans la poche. Nina s'assoit sur le seuil. C'est son voyage. Oui. Merci, l'herbe garde son voyage. La vitre de la porte montre le banc, net. Le cartable est chaud, contre la jambe. Le chemin attend, large et pâle.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La veine d'herbe reste sur le papier, dans la poche. Nina s'assoit sur le seuil. C'est son voyage. Oui. Merci de l'avoir laissée. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; de la porte montre le banc, net. Le cartable est chaud, contre la jambe. Le chemin attend, large et pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La veine d'herbe reste sur le papier, dans la poche. Nina s'assoit sur le seuil. C'est son voyage. Oui. Merci, l'herbe garde son voyage. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; de la porte montre le banc, net. Le cartable est chaud, contre la jambe. Le chemin attend, large et pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La veine d'herbe reste sur le papier, dans la poche. Nina s'assoit sur le seuil. C'est son voyage. Oui. Merci de l'avoir laissée. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; de la porte montre le banc, net. Le cartable est chaud, contre la jambe. Le chemin attend, large et pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La veine d'herbe reste sur le papier, dans la poche. Nina s'assoit sur le seuil. C'est son voyage. Oui. Merci, l'herbe garde son voyage. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; de la porte montre le banc, net. Le cartable est chaud, contre la jambe. Le chemin attend, large et pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10222,7 +10222,7 @@
 narrateur|Nina s'assoit sur le seuil.
 enfant-f|C'est son voyage.
 papa|Oui.
-maman|Merci de l'avoir laissée.
+maman|Merci, l'herbe garde son voyage.
 narrateur|La vitre de la porte montre le banc, net.
 narrateur|Le cartable est chaud, contre la jambe.
 narrateur|Le chemin attend, large et pâle.</t>
@@ -10442,17 +10442,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Plus de papillon au verre. Contre le carton, le dessin dort. Bonjour, haie. Elle ne répond pas, c'est normal. Merci d'avoir parlé sans ouvrir. Le cartable est dans la maison, sentant le thym. La porte du jardin est noire, un peu froide. Une aile a laissé une poussière d'or, minuscule.</t>
+          <t>Plus de papillon au verre. Contre le carton, le dessin dort. Bonjour, haie. Elle ne répond pas, c'est normal. Merci, le papillon a eu sa phrase. Le cartable est dans la maison, sentant le thym. La porte du jardin est noire, un peu froide. Une aile a laissé une poussière d'or, minuscule.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus de papillon au verre. Contre le carton, le dessin dort. Bonjour, haie. Elle ne répond pas, c'est normal. Merci d'avoir parlé sans ouvrir. Le cartable est dans la maison, sentant le thym. La porte du jardin est noire, un peu froide. Une aile a laissé une poussière d'or, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus de papillon au verre. Contre le carton, le dessin dort. Bonjour, haie. Elle ne répond pas, c'est normal. Merci, le papillon a eu sa phrase. Le cartable est dans la maison, sentant le thym. La porte du jardin est noire, un peu froide. Une aile a laissé une poussière d'or, minuscule.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus de papillon au verre. Contre le carton, le dessin dort. Bonjour, haie. Elle ne répond pas, c'est normal. Merci d'avoir parlé sans ouvrir. Le cartable est dans la maison, sentant le thym. La porte du jardin est noire, un peu froide. Une aile a laissé une poussière d'or, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus de papillon au verre. Contre le carton, le dessin dort. Bonjour, haie. Elle ne répond pas, c'est normal. Merci, le papillon a eu sa phrase. Le cartable est dans la maison, sentant le thym. La porte du jardin est noire, un peu froide. Une aile a laissé une poussière d'or, minuscule.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10594,7 +10594,7 @@
 narrateur|Contre le carton, le dessin dort.
 enfant-f|Bonjour, haie.
 maman|Elle ne répond pas, c'est normal.
-papa|Merci d'avoir parlé sans ouvrir.
+papa|Merci, le papillon a eu sa phrase.
 narrateur|Le cartable est dans la maison, sentant le thym.
 narrateur|La porte du jardin est noire, un peu froide.
 narrateur|Une aile a laissé une poussière d'or, minuscule.</t>
@@ -11201,17 +11201,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Nina a le cartable sur les épaules, un bras, puis l'autre. Le torchon flotte un peu, sur la corde. Ça ne glisse plus. La courroie est sèche. Merci d'avoir demandé l'aide. Les dalles sont claires, vides. Le chemin prend le jaune et l'emmène. Le crochet ne pend plus rien.</t>
+          <t>Nina a le cartable sur les épaules, un bras, puis l'autre. Le torchon flotte un peu, sur la corde. Ça ne glisse plus. La courroie est sèche. Merci, tes épaules sont prêtes. Les dalles sont claires, vides. Le chemin prend le jaune et l'emmène. Le crochet ne pend plus rien.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina a le cartable sur les épaules, un bras, puis l'autre. Le torchon flotte un peu, sur la corde. Ça ne glisse plus. La courroie est sèche. Merci d'avoir demandé l'aide. Les dalles sont claires, vides. Le chemin prend le jaune et l'emmène. Le crochet ne pend plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina a le cartable sur les épaules, un bras, puis l'autre. Le torchon flotte un peu, sur la corde. Ça ne glisse plus. La courroie est sèche. Merci, tes épaules sont prêtes. Les dalles sont claires, vides. Le chemin prend le jaune et l'emmène. Le crochet ne pend plus rien.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina a le cartable sur les épaules, un bras, puis l'autre. Le torchon flotte un peu, sur la corde. Ça ne glisse plus. La courroie est sèche. Merci d'avoir demandé l'aide. Les dalles sont claires, vides. Le chemin prend le jaune et l'emmène. Le crochet ne pend plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina a le cartable sur les épaules, un bras, puis l'autre. Le torchon flotte un peu, sur la corde. Ça ne glisse plus. La courroie est sèche. Merci, tes épaules sont prêtes. Les dalles sont claires, vides. Le chemin prend le jaune et l'emmène. Le crochet ne pend plus rien.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11353,7 +11353,7 @@
 narrateur|Le torchon flotte un peu, sur la corde.
 enfant-f|Ça ne glisse plus.
 papa|La courroie est sèche.
-maman|Merci d'avoir demandé l'aide.
+maman|Merci, tes épaules sont prêtes.
 narrateur|Les dalles sont claires, vides.
 narrateur|Le chemin prend le jaune et l'emmène.
 narrateur|Le crochet ne pend plus rien.</t>
@@ -11574,17 +11574,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Le torchon est sur la marche, plié. Le cartable dort contre le mur, à l'ombre. Le lézard est parti. Oui. Merci d'avoir choisi la marche. Les dalles tiennent les pieds, sans glisser. Une feuille sèche tremble, puis s'arrête. Le jaune du mur est plus pâle que le sac.</t>
+          <t>Le torchon est sur la marche, plié. Le cartable dort contre le mur, à l'ombre. Le lézard est parti. Oui. Merci, la marche le garde. Les dalles tiennent les pieds, sans glisser. Une feuille sèche tremble, puis s'arrête. Le jaune du mur est plus pâle que le sac.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le torchon est sur la marche, plié. Le cartable dort contre le mur, à l'ombre. Le lézard est parti. Oui. Merci d'avoir choisi la marche. Les dalles tiennent les pieds, sans glisser. Une feuille sèche tremble, puis s'arrête. Le jaune du mur est plus pâle que le sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le torchon est sur la marche, plié. Le cartable dort contre le mur, à l'ombre. Le lézard est parti. Oui. Merci, la marche le garde. Les dalles tiennent les pieds, sans glisser. Une feuille sèche tremble, puis s'arrête. Le jaune du mur est plus pâle que le sac.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le torchon est sur la marche, plié. Le cartable dort contre le mur, à l'ombre. Le lézard est parti. Oui. Merci d'avoir choisi la marche. Les dalles tiennent les pieds, sans glisser. Une feuille sèche tremble, puis s'arrête. Le jaune du mur est plus pâle que le sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le torchon est sur la marche, plié. Le cartable dort contre le mur, à l'ombre. Le lézard est parti. Oui. Merci, la marche le garde. Les dalles tiennent les pieds, sans glisser. Une feuille sèche tremble, puis s'arrête. Le jaune du mur est plus pâle que le sac.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11726,7 +11726,7 @@
 narrateur|Le cartable dort contre le mur, à l'ombre.
 enfant-f|Le lézard est parti.
 maman|Oui.
-papa|Merci d'avoir choisi la marche.
+papa|Merci, la marche le garde.
 narrateur|Les dalles tiennent les pieds, sans glisser.
 narrateur|Une feuille sèche tremble, puis s'arrête.
 narrateur|Le jaune du mur est plus pâle que le sac.</t>
@@ -11945,17 +11945,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Le cartable rentre, sentant le jardin et le torchon. Un rond de lampe reste sur la porte. Le crochet est vide. Oui. Merci d'avoir tenu le sac. Nina a les doigts un peu rèches, de la toile. La nuit a pris le chemin. Le jaune est à l'intérieur, enfin.</t>
+          <t>Le cartable rentre, sentant le jardin et le torchon. Un rond de lampe reste sur la porte. Le crochet est vide. Oui. Merci, le sac est rentré. Nina a les doigts un peu rèches, de la toile. La nuit a pris le chemin. Le jaune est à l'intérieur, enfin.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable rentre, sentant le jardin et le torchon. Un rond de lampe reste sur la porte. Le crochet est vide. Oui. Merci d'avoir tenu le sac. Nina a les doigts un peu rèches, de la toile. La nuit a pris le chemin. Le jaune est à l'intérieur, enfin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable rentre, sentant le jardin et le torchon. Un rond de lampe reste sur la porte. Le crochet est vide. Oui. Merci, le sac est rentré. Nina a les doigts un peu rèches, de la toile. La nuit a pris le chemin. Le jaune est à l'intérieur, enfin.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable rentre, sentant le jardin et le torchon. Un rond de lampe reste sur la porte. Le crochet est vide. Oui. Merci d'avoir tenu le sac. Nina a les doigts un peu rèches, de la toile. La nuit a pris le chemin. Le jaune est à l'intérieur, enfin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable rentre, sentant le jardin et le torchon. Un rond de lampe reste sur la porte. Le crochet est vide. Oui. Merci, le sac est rentré. Nina a les doigts un peu rèches, de la toile. La nuit a pris le chemin. Le jaune est à l'intérieur, enfin.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12097,7 +12097,7 @@
 narrateur|Un rond de lampe reste sur la porte.
 enfant-f|Le crochet est vide.
 papa|Oui.
-maman|Merci d'avoir tenu le sac.
+maman|Merci, le sac est rentré.
 narrateur|Nina a les doigts un peu rèches, de la toile.
 narrateur|La nuit a pris le chemin.
 narrateur|Le jaune est à l'intérieur, enfin.</t>
@@ -13460,17 +13460,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Nina quitte la chambre, le cartable un peu lourd. Le pull garde son creux, sur le lit. Les chaussettes sont chaudes. Oui. Merci d'avoir attendu. La vitre montre le chemin, sans buée. La chaise est vide, un peu chaude. La boîte tape le dos, toc, vers l'école.</t>
+          <t>Nina quitte la chambre, le cartable un peu lourd. Le pull garde son creux, sur le lit. Les chaussettes sont chaudes. Oui. Merci, on peut partir. La vitre montre le chemin, sans buée. La chaise est vide, un peu chaude. La boîte tape le dos, toc, vers l'école.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina quitte la chambre, le cartable un peu lourd. Le pull garde son creux, sur le lit. Les chaussettes sont chaudes. Oui. Merci d'avoir attendu. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; montre le chemin, sans buée. La chaise est vide, un peu chaude. La boîte tape le dos, toc, vers l'école.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina quitte la chambre, le cartable un peu lourd. Le pull garde son creux, sur le lit. Les chaussettes sont chaudes. Oui. Merci, on peut partir. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; montre le chemin, sans buée. La chaise est vide, un peu chaude. La boîte tape le dos, toc, vers l'école.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina quitte la chambre, le cartable un peu lourd. Le pull garde son creux, sur le lit. Les chaussettes sont chaudes. Oui. Merci d'avoir attendu. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; montre le chemin, sans buée. La chaise est vide, un peu chaude. La boîte tape le dos, toc, vers l'école.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina quitte la chambre, le cartable un peu lourd. Le pull garde son creux, sur le lit. Les chaussettes sont chaudes. Oui. Merci, on peut partir. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; montre le chemin, sans buée. La chaise est vide, un peu chaude. La boîte tape le dos, toc, vers l'école.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13612,7 +13612,7 @@
 narrateur|Le pull garde son creux, sur le lit.
 enfant-f|Les chaussettes sont chaudes.
 maman|Oui.
-papa|Merci d'avoir attendu.
+papa|Merci, on peut partir.
 narrateur|La vitre montre le chemin, sans buée.
 narrateur|La chaise est vide, un peu chaude.
 narrateur|La boîte tape le dos, toc, vers l'école.</t>
@@ -13832,17 +13832,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Nina écoute le toc, au fond du cartable. La boîte est là, pour plus tard. Je l'ai entendue. Moi aussi. Merci d'avoir demandé avant de sortir. L'oreiller reprend sa forme, lentement. Un grain de soleil tient sur la fermeture. La chaise garde le jaune, comme un ami.</t>
+          <t>Nina écoute le toc, au fond du cartable. La boîte est là, pour plus tard. Je l'ai entendue. Moi aussi. Merci, on l'entend bien. L'oreiller reprend sa forme, lentement. Un grain de soleil tient sur la fermeture. La chaise garde le jaune, comme un ami.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina écoute le toc, au fond du cartable. La boîte est là, pour plus tard. Je l'ai entendue. Moi aussi. Merci d'avoir demandé avant de sortir. L'oreiller reprend sa forme, lentement. Un grain de soleil tient sur la fermeture. La chaise garde le jaune, comme un ami.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nina écoute le toc, au fond du cartable. La boîte est là, pour plus tard. Je l'ai entendue. Moi aussi. Merci, on l'entend bien. L'oreiller reprend sa forme, lentement. Un grain de soleil tient sur la fermeture. La chaise garde le jaune, comme un ami.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina écoute le toc, au fond du cartable. La boîte est là, pour plus tard. Je l'ai entendue. Moi aussi. Merci d'avoir demandé avant de sortir. L'oreiller reprend sa forme, lentement. Un grain de soleil tient sur la fermeture. La chaise garde le jaune, comme un ami.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nina écoute le toc, au fond du cartable. La boîte est là, pour plus tard. Je l'ai entendue. Moi aussi. Merci, on l'entend bien. L'oreiller reprend sa forme, lentement. Un grain de soleil tient sur la fermeture. La chaise garde le jaune, comme un ami.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13984,7 +13984,7 @@
 narrateur|La boîte est là, pour plus tard.
 enfant-f|Je l'ai entendue.
 papa|Moi aussi.
-maman|Merci d'avoir demandé avant de sortir.
+maman|Merci, on l'entend bien.
 narrateur|L'oreiller reprend sa forme, lentement.
 narrateur|Un grain de soleil tient sur la fermeture.
 narrateur|La chaise garde le jaune, comme un ami.</t>
@@ -14203,17 +14203,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Une miette a goûté le soir, une seule. La boîte est refermée. Demain. Demain. Merci d'avoir refermé. La veilleuse tient le cartable d'or. Le verre de la chambre est une nuit calme. Le pull, sur le lit, n'a plus de secret.</t>
+          <t>Une miette a goûté le soir, une seule. La boîte est refermée. Demain. Demain. Merci, la boîte est close. La veilleuse tient le cartable d'or. Le verre de la chambre est une nuit calme. Le pull, sur le lit, n'a plus de secret.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une miette a goûté le soir, une seule. La boîte est refermée. Demain. Demain. Merci d'avoir refermé. La veilleuse tient le cartable d'or. Le verre de la chambre est une nuit calme. Le pull, sur le lit, n'a plus de secret.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Une miette a goûté le soir, une seule. La boîte est refermée. Demain. Demain. Merci, la boîte est close. La veilleuse tient le cartable d'or. Le verre de la chambre est une nuit calme. Le pull, sur le lit, n'a plus de secret.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une miette a goûté le soir, une seule. La boîte est refermée. Demain. Demain. Merci d'avoir refermé. La veilleuse tient le cartable d'or. Le verre de la chambre est une nuit calme. Le pull, sur le lit, n'a plus de secret.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Une miette a goûté le soir, une seule. La boîte est refermée. Demain. Demain. Merci, la boîte est close. La veilleuse tient le cartable d'or. Le verre de la chambre est une nuit calme. Le pull, sur le lit, n'a plus de secret.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14355,7 +14355,7 @@
 narrateur|La boîte est refermée.
 enfant-f|Demain.
 maman|Demain.
-papa|Merci d'avoir refermé.
+papa|Merci, la boîte est close.
 narrateur|La veilleuse tient le cartable d'or.
 narrateur|Le verre de la chambre est une nuit calme.
 narrateur|Le pull, sur le lit, n'a plus de secret.</t>
@@ -14962,17 +14962,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>La cloche lointaine a fini. La maison jaune voyage dans la poche. Elle n'est plus sous le lit. Non. Merci d'avoir demandé la poche. La chaussette reste seule, sous le bois. La chaise est vide. Le chemin entre dans les yeux de Nina, clair.</t>
+          <t>La cloche lointaine a fini. La maison jaune voyage dans la poche. Elle n'est plus sous le lit. C'est vrai. Merci, la poche la garde. La chaussette reste seule, sous le bois. La chaise est vide. Le chemin entre dans les yeux de Nina, clair.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La cloche lointaine a fini. La maison jaune voyage dans la poche. Elle n'est plus sous le lit. Non. Merci d'avoir demandé la poche. La chaussette reste seule, sous le bois. La chaise est vide. Le chemin entre dans les yeux de Nina, clair.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La cloche lointaine a fini. La maison jaune voyage dans la poche. Elle n'est plus sous le lit. C'est vrai. Merci, la poche la garde. La chaussette reste seule, sous le bois. La chaise est vide. Le chemin entre dans les yeux de Nina, clair.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La cloche lointaine a fini. La maison jaune voyage dans la poche. Elle n'est plus sous le lit. Non. Merci d'avoir demandé la poche. La chaussette reste seule, sous le bois. La chaise est vide. Le chemin entre dans les yeux de Nina, clair.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La cloche lointaine a fini. La maison jaune voyage dans la poche. Elle n'est plus sous le lit. C'est vrai. Merci, la poche la garde. La chaussette reste seule, sous le bois. La chaise est vide. Le chemin entre dans les yeux de Nina, clair.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15113,8 +15113,8 @@
           <t>narrateur|La cloche lointaine a fini.
 narrateur|La maison jaune voyage dans la poche.
 enfant-f|Elle n'est plus sous le lit.
-papa|Non.
-maman|Merci d'avoir demandé la poche.
+papa|C'est vrai.
+maman|Merci, la poche la garde.
 narrateur|La chaussette reste seule, sous le bois.
 narrateur|La chaise est vide.
 narrateur|Le chemin entre dans les yeux de Nina, clair.</t>
@@ -15334,17 +15334,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>La poussière est retombée. Le dessin est dans la poche, tiède. Pas à la vitre, dans le sac. Oui. Merci d'avoir choisi. Le cartable, sur la chaise, a l'air prêt. Un dernier grain brille, puis plus rien. Le chemin, dehors, attend sans frapper au verre.</t>
+          <t>La poussière est retombée. Le dessin est dans la poche, tiède. Pas à la vitre, dans le sac. Oui. Merci, la poche a gagné. Le cartable, sur la chaise, a l'air prêt. Un dernier grain brille, puis plus rien. Le chemin, dehors, attend sans frapper au verre.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poussière est retombée. Le dessin est dans la poche, tiède. Pas à la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt;, dans le sac. Oui. Merci d'avoir choisi. Le cartable, sur la chaise, a l'air prêt. Un dernier grain brille, puis plus rien. Le chemin, dehors, attend sans frapper au verre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poussière est retombée. Le dessin est dans la poche, tiède. Pas à la &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt;, dans le sac. Oui. Merci, la poche a gagné. Le cartable, sur la chaise, a l'air prêt. Un dernier grain brille, puis plus rien. Le chemin, dehors, attend sans frapper au verre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poussière est retombée. Le dessin est dans la poche, tiède. Pas à la &lt;emphasis&gt;vitre&lt;/emphasis&gt;, dans le sac. Oui. Merci d'avoir choisi. Le cartable, sur la chaise, a l'air prêt. Un dernier grain brille, puis plus rien. Le chemin, dehors, attend sans frapper au verre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poussière est retombée. Le dessin est dans la poche, tiède. Pas à la &lt;emphasis&gt;vitre&lt;/emphasis&gt;, dans le sac. Oui. Merci, la poche a gagné. Le cartable, sur la chaise, a l'air prêt. Un dernier grain brille, puis plus rien. Le chemin, dehors, attend sans frapper au verre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15486,7 +15486,7 @@
 narrateur|Le dessin est dans la poche, tiède.
 enfant-f|Pas à la vitre, dans le sac.
 maman|Oui.
-papa|Merci d'avoir choisi.
+papa|Merci, la poche a gagné.
 narrateur|Le cartable, sur la chaise, a l'air prêt.
 narrateur|Un dernier grain brille, puis plus rien.
 narrateur|Le chemin, dehors, attend sans frapper au verre.</t>
@@ -16464,17 +16464,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>L'ovale en forme de maison cadre le chemin. Nina ne frotte plus. Si je frotte, il part. Oui. Merci de t'être arrêtée. Le torchon reste sur le radiateur, inutile. Le cartable quitte la chaise, jaune et net. Le tic du radiateur s'est tu.</t>
+          <t>L'ovale en forme de maison cadre le chemin. Nina ne frotte plus. Si je frotte, il part. Oui. Merci, l'ovale reste. Le torchon reste sur le radiateur, inutile. Le cartable quitte la chaise, jaune et net. Le tic du radiateur s'est tu.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'ovale en forme de maison cadre le chemin. Nina ne frotte plus. Si je frotte, il part. Oui. Merci de t'être arrêtée. Le torchon reste sur le radiateur, inutile. Le cartable quitte la chaise, jaune et net. Le tic du radiateur s'est tu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'ovale en forme de maison cadre le chemin. Nina ne frotte plus. Si je frotte, il part. Oui. Merci, l'ovale reste. Le torchon reste sur le radiateur, inutile. Le cartable quitte la chaise, jaune et net. Le tic du radiateur s'est tu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'ovale en forme de maison cadre le chemin. Nina ne frotte plus. Si je frotte, il part. Oui. Merci de t'être arrêtée. Le torchon reste sur le radiateur, inutile. Le cartable quitte la chaise, jaune et net. Le tic du radiateur s'est tu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'ovale en forme de maison cadre le chemin. Nina ne frotte plus. Si je frotte, il part. Oui. Merci, l'ovale reste. Le torchon reste sur le radiateur, inutile. Le cartable quitte la chaise, jaune et net. Le tic du radiateur s'est tu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16616,7 +16616,7 @@
 narrateur|Nina ne frotte plus.
 enfant-f|Si je frotte, il part.
 maman|Oui.
-papa|Merci de t'être arrêtée.
+papa|Merci, l'ovale reste.
 narrateur|Le torchon reste sur le radiateur, inutile.
 narrateur|Le cartable quitte la chaise, jaune et net.
 narrateur|Le tic du radiateur s'est tu.</t>
@@ -16836,17 +16836,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Le cartable n'est plus un chat, il est sur le dos. Le radiateur fait un dernier tic. Il était prêt. Oui. Merci d'avoir demandé qu'on le tende. Le torchon n'a plus de travail. Un rayon a quitté la boucle. La vitre sèche garde le chemin, sans ovale.</t>
+          <t>Le cartable n'est plus un chat, il est sur le dos. Le radiateur fait un dernier tic. Il était prêt. Oui. Merci, il est à toi. Le torchon n'a plus de travail. Un rayon a quitté la boucle. La vitre sèche garde le chemin, sans ovale.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable n'est plus un chat, il est sur le dos. Le radiateur fait un dernier tic. Il était prêt. Oui. Merci d'avoir demandé qu'on le tende. Le torchon n'a plus de travail. Un rayon a quitté la boucle. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; sèche garde le chemin, sans ovale.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable n'est plus un chat, il est sur le dos. Le radiateur fait un dernier tic. Il était prêt. Oui. Merci, il est à toi. Le torchon n'a plus de travail. Un rayon a quitté la boucle. La &lt;emphasis level="moderate"&gt;vitre&lt;/emphasis&gt; sèche garde le chemin, sans ovale.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable n'est plus un chat, il est sur le dos. Le radiateur fait un dernier tic. Il était prêt. Oui. Merci d'avoir demandé qu'on le tende. Le torchon n'a plus de travail. Un rayon a quitté la boucle. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; sèche garde le chemin, sans ovale.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable n'est plus un chat, il est sur le dos. Le radiateur fait un dernier tic. Il était prêt. Oui. Merci, il est à toi. Le torchon n'a plus de travail. Un rayon a quitté la boucle. La &lt;emphasis&gt;vitre&lt;/emphasis&gt; sèche garde le chemin, sans ovale.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -16988,7 +16988,7 @@
 narrateur|Le radiateur fait un dernier tic.
 enfant-f|Il était prêt.
 papa|Oui.
-maman|Merci d'avoir demandé qu'on le tende.
+maman|Merci, il est à toi.
 narrateur|Le torchon n'a plus de travail.
 narrateur|Un rayon a quitté la boucle.
 narrateur|La vitre sèche garde le chemin, sans ovale.</t>
@@ -17388,7 +17388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17445,6 +17445,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>